<commit_message>
add frontend/backend for hardware analyzing
</commit_message>
<xml_diff>
--- a/Symptom_Rootcause_Ticket_Evaluation/output/AI Jira Bug to Symptom Assignment validation.xlsx
+++ b/Symptom_Rootcause_Ticket_Evaluation/output/AI Jira Bug to Symptom Assignment validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dentsplysirona-my.sharepoint.com/personal/christian_kurz_dentsplysirona_com/Documents/_IO-Sensor/10_Qualität/05_Feld/99_Siroforce/00_Git/Y3839-IO_Workspace/Symptom_Rootcause_Ticket_Evaluation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="8_{236449CA-312A-4DB1-B587-EDE847815BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A151186D-7EB7-4616-A052-C1630698C4DA}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="8_{236449CA-312A-4DB1-B587-EDE847815BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2748B234-A9BD-4C9E-B799-33741C4BDE39}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52E5B530-6EC2-40DF-B8D2-2FAAD7B66627}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="282">
   <si>
     <t>Column1</t>
   </si>
@@ -341,18 +341,33 @@
     <t>Michael</t>
   </si>
   <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>IOSS not installed</t>
+  </si>
+  <si>
     <t>Y3839-710</t>
   </si>
   <si>
     <t>Remote Box is not usable after reinstall of IOSS/CDR Drivers</t>
   </si>
   <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>cannot be categorized, IOSS driver reinstallation</t>
+  </si>
+  <si>
     <t>Y3839-307</t>
   </si>
   <si>
     <t>Sensor upgrading fails for XIOS XG</t>
   </si>
   <si>
+    <t>Sensor upgrading not implemented</t>
+  </si>
+  <si>
     <t>Y3839-506</t>
   </si>
   <si>
@@ -365,24 +380,36 @@
     <t>Only one firmware available for XIOS XG Supreme/Schick 33 sensors</t>
   </si>
   <si>
+    <t>Only one sensor firmware</t>
+  </si>
+  <si>
     <t>Y3839-611</t>
   </si>
   <si>
     <t xml:space="preserve"> FirmwareUpgradeUtility is sending commands when an USB Stick is connected </t>
   </si>
   <si>
+    <t>Firmware Upgrader bug</t>
+  </si>
+  <si>
     <t>Y3839-625</t>
   </si>
   <si>
     <t>GETFPGAVersions returns null after successful flash</t>
   </si>
   <si>
+    <t>FPGA flash erase issue</t>
+  </si>
+  <si>
     <t>Y3839-661</t>
   </si>
   <si>
     <t>SensorConnected property does not update in Upgrade State</t>
   </si>
   <si>
+    <t>FW bug</t>
+  </si>
+  <si>
     <t>Y3839-689</t>
   </si>
   <si>
@@ -395,12 +422,21 @@
     <t>Indication region in Sidexis is different to the one in indication dialog</t>
   </si>
   <si>
+    <t>cannot be categorized, Docu bug / IOSS bug</t>
+  </si>
+  <si>
     <t>Y3839-705</t>
   </si>
   <si>
     <t>IOSS Installer: Error Text Stays German Even if other languages is selected</t>
   </si>
   <si>
+    <t xml:space="preserve">no </t>
+  </si>
+  <si>
+    <t>cannot be categorized, IOSS Installer bug</t>
+  </si>
+  <si>
     <t>Y3839-711</t>
   </si>
   <si>
@@ -413,6 +449,9 @@
     <t>Applicable standards missing</t>
   </si>
   <si>
+    <t xml:space="preserve">cannot be categorized, Docu bug  </t>
+  </si>
+  <si>
     <t>Y3839-718</t>
   </si>
   <si>
@@ -467,9 +506,6 @@
     <t>Loose micro-B USB interface (no cable clip used)</t>
   </si>
   <si>
-    <t>yes</t>
-  </si>
-  <si>
     <t>Y3839-265</t>
   </si>
   <si>
@@ -479,9 +515,6 @@
     <t>Loose USB3 remote/sensor interface</t>
   </si>
   <si>
-    <t>no</t>
-  </si>
-  <si>
     <t>cannot be categorized, LED sequence is due to the boot process</t>
   </si>
   <si>
@@ -569,7 +602,7 @@
     <t>Sensor stays unregistered in Sidexis after 401 on device re-registration (expired refresh token, no retry)</t>
   </si>
   <si>
-    <t>Intermittent Connectivity -&gt; IOSS bugs ?</t>
+    <t>IOSS bug?</t>
   </si>
   <si>
     <t>Y3839-231</t>
@@ -596,6 +629,9 @@
     <t>Sidexis/IOSS: Viewport remains red after sensor reconnect, sensor shown twice in configuration app and Sidexis</t>
   </si>
   <si>
+    <t>Intermittent Connectivity -&gt; Missing Error handling in SW/FW</t>
+  </si>
+  <si>
     <t>Y3839-575</t>
   </si>
   <si>
@@ -695,9 +731,6 @@
     <t>Broken FPGA image still loaded after sensor unplugged</t>
   </si>
   <si>
-    <t>FW bug</t>
-  </si>
-  <si>
     <t>Y3839-712</t>
   </si>
   <si>
@@ -725,12 +758,18 @@
     <t/>
   </si>
   <si>
+    <t>graphic (positioning holder) missing in Sidexis</t>
+  </si>
+  <si>
     <t>Y3839-309</t>
   </si>
   <si>
     <t>Unsupported language template list output inconsistently translated</t>
   </si>
   <si>
+    <t>translation issue in Sidexis</t>
+  </si>
+  <si>
     <t>Y3839-340</t>
   </si>
   <si>
@@ -761,6 +800,9 @@
     <t>X-ray tab in Intraoral Config app only support German and English</t>
   </si>
   <si>
+    <t>translation issue in Intraoral Config App</t>
+  </si>
+  <si>
     <t>Y3839-513</t>
   </si>
   <si>
@@ -797,10 +839,16 @@
     <t>Odontogram in indication dialog is active only if it's not predefined in viewset</t>
   </si>
   <si>
+    <t>documentation mismatch</t>
+  </si>
+  <si>
     <t>Y3839-709</t>
   </si>
   <si>
     <t>Endo horizontal and endo vertical templates do not contain predefined anatomic regions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not assigned </t>
   </si>
   <si>
     <t>Y3839-734</t>
@@ -1309,7 +1357,7 @@
     <col min="3" max="3" width="52.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="66.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="49.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1339,7 +1387,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="29.25">
+    <row r="2" spans="1:8" ht="30">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1660,7 +1708,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>60</v>
       </c>
@@ -1677,7 +1725,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>63</v>
       </c>
@@ -1694,7 +1742,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -1711,7 +1759,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>67</v>
       </c>
@@ -1728,7 +1776,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -1745,7 +1793,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1762,7 +1810,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -1779,7 +1827,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -1796,7 +1844,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>78</v>
       </c>
@@ -1813,7 +1861,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>80</v>
       </c>
@@ -1830,7 +1878,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>82</v>
       </c>
@@ -1847,7 +1895,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -1864,7 +1912,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -1881,7 +1929,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>88</v>
       </c>
@@ -1898,7 +1946,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>90</v>
       </c>
@@ -1914,13 +1962,19 @@
       <c r="E31" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31" t="s">
+        <v>95</v>
+      </c>
+      <c r="G31" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
         <v>92</v>
@@ -1931,13 +1985,19 @@
       <c r="E32" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="F32" t="s">
+        <v>99</v>
+      </c>
+      <c r="G32" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B33" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C33" t="s">
         <v>92</v>
@@ -1948,13 +2008,19 @@
       <c r="E33" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33" t="s">
+        <v>95</v>
+      </c>
+      <c r="G33" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B34" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C34" t="s">
         <v>92</v>
@@ -1965,13 +2031,19 @@
       <c r="E34" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="F34" t="s">
+        <v>95</v>
+      </c>
+      <c r="G34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B35" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C35" t="s">
         <v>92</v>
@@ -1982,13 +2054,19 @@
       <c r="E35" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35" t="s">
+        <v>95</v>
+      </c>
+      <c r="G35" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B36" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C36" t="s">
         <v>92</v>
@@ -1999,13 +2077,19 @@
       <c r="E36" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="F36" t="s">
+        <v>95</v>
+      </c>
+      <c r="G36" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B37" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C37" t="s">
         <v>92</v>
@@ -2016,13 +2100,19 @@
       <c r="E37" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="F37" t="s">
+        <v>95</v>
+      </c>
+      <c r="G37" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B38" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C38" t="s">
         <v>92</v>
@@ -2033,13 +2123,19 @@
       <c r="E38" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="F38" t="s">
+        <v>95</v>
+      </c>
+      <c r="G38" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="B39" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C39" t="s">
         <v>92</v>
@@ -2050,13 +2146,19 @@
       <c r="E39" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="F39" t="s">
+        <v>95</v>
+      </c>
+      <c r="G39" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="B40" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C40" t="s">
         <v>92</v>
@@ -2067,13 +2169,19 @@
       <c r="E40" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="F40" t="s">
+        <v>99</v>
+      </c>
+      <c r="G40" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B41" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="C41" t="s">
         <v>92</v>
@@ -2084,13 +2192,19 @@
       <c r="E41" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="F41" t="s">
+        <v>125</v>
+      </c>
+      <c r="G41" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="B42" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="C42" t="s">
         <v>92</v>
@@ -2101,13 +2215,19 @@
       <c r="E42" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="F42" t="s">
+        <v>95</v>
+      </c>
+      <c r="G42" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="B43" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C43" t="s">
         <v>92</v>
@@ -2118,606 +2238,621 @@
       <c r="E43" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="F43" t="s">
+        <v>99</v>
+      </c>
+      <c r="G43" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B44" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C44" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D44" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="E44" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="B45" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C45" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="E45" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="B46" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="C46" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D46" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="E46" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="B47" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="C47" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D47" t="s">
         <v>32</v>
       </c>
       <c r="E47" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="B48" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C48" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D48" t="s">
         <v>32</v>
       </c>
       <c r="E48" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
+        <v>147</v>
+      </c>
+      <c r="B49" t="s">
+        <v>148</v>
+      </c>
+      <c r="C49" t="s">
         <v>134</v>
       </c>
-      <c r="B49" t="s">
-        <v>135</v>
-      </c>
-      <c r="C49" t="s">
-        <v>121</v>
-      </c>
       <c r="D49" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="E49" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F49" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B50" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C50" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D50" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="E50" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F50" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="G50" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:7">
       <c r="A51" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="C51" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D51" t="s">
         <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F51" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="B52" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C52" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D52" t="s">
         <v>24</v>
       </c>
       <c r="E52" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F52" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:7">
       <c r="A53" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="B53" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="C53" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D53" t="s">
         <v>24</v>
       </c>
       <c r="E53" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F53" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:7">
       <c r="A54" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="B54" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="C54" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D54" t="s">
         <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F54" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:7">
       <c r="A55" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="B55" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="C55" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D55" t="s">
         <v>24</v>
       </c>
       <c r="E55" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F55" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="B56" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="C56" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D56" t="s">
         <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F56" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="G56" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="B57" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="C57" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D57" t="s">
         <v>24</v>
       </c>
       <c r="E57" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F57" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="B58" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="C58" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D58" t="s">
         <v>24</v>
       </c>
       <c r="E58" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F58" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B59" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="C59" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D59" t="s">
         <v>24</v>
       </c>
       <c r="E59" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F59" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="G59" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:7">
       <c r="A60" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="B60" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C60" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D60" t="s">
         <v>24</v>
       </c>
       <c r="E60" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F60" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="61" spans="1:7">
       <c r="A61" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="B61" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C61" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D61" t="s">
         <v>24</v>
       </c>
       <c r="E61" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F61" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62" spans="1:7">
       <c r="A62" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="B62" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="C62" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D62" t="s">
         <v>24</v>
       </c>
       <c r="E62" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F62" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="63" spans="1:7">
       <c r="A63" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="B63" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="C63" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D63" t="s">
         <v>24</v>
       </c>
       <c r="E63" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F63" t="s">
-        <v>141</v>
+        <v>95</v>
       </c>
       <c r="G63" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
     </row>
     <row r="64" spans="1:7">
       <c r="A64" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="B64" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="C64" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D64" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E64" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F64" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="B65" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="C65" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D65" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E65" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="B66" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="C66" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D66" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E66" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F66" t="s">
+        <v>99</v>
+      </c>
+      <c r="G66" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="B67" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="C67" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D67" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E67" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F67" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:7">
       <c r="A68" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="B68" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C68" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D68" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E68" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="B69" t="s">
+        <v>197</v>
+      </c>
+      <c r="C69" t="s">
+        <v>134</v>
+      </c>
+      <c r="D69" t="s">
         <v>185</v>
       </c>
-      <c r="C69" t="s">
-        <v>121</v>
-      </c>
-      <c r="D69" t="s">
-        <v>174</v>
-      </c>
       <c r="E69" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="B70" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="C70" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D70" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E70" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="B71" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C71" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="D71" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="E71" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:7">
       <c r="A72" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="B72" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="C72" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
       </c>
       <c r="E72" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="B73" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="C73" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="D73" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="E73" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
     </row>
     <row r="74" spans="1:7">
       <c r="A74" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="B74" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C74" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="D74" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="E74" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="B75" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C75" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D75" t="s">
         <v>24</v>
@@ -2729,18 +2864,18 @@
         <v>26</v>
       </c>
       <c r="G75" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="B76" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="C76" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D76" t="s">
         <v>24</v>
@@ -2752,18 +2887,18 @@
         <v>26</v>
       </c>
       <c r="G76" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="B77" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C77" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D77" t="s">
         <v>24</v>
@@ -2775,327 +2910,363 @@
         <v>92</v>
       </c>
       <c r="G77" t="s">
-        <v>213</v>
+        <v>117</v>
       </c>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="B78" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="C78" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D78" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="E78" t="s">
         <v>25</v>
       </c>
       <c r="F78" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="G78" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="B79" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="C79" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D79" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E79" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F79" t="s">
+        <v>228</v>
+      </c>
+      <c r="G79" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="B80" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="C80" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D80" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E80" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F80" t="s">
+        <v>228</v>
+      </c>
+      <c r="G80" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="B81" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C81" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D81" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E81" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F81" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="G81" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="B82" t="s">
+        <v>241</v>
+      </c>
+      <c r="C82" t="s">
+        <v>232</v>
+      </c>
+      <c r="D82" t="s">
+        <v>233</v>
+      </c>
+      <c r="E82" t="s">
+        <v>136</v>
+      </c>
+      <c r="F82" t="s">
         <v>228</v>
       </c>
-      <c r="C82" t="s">
-        <v>221</v>
-      </c>
-      <c r="D82" t="s">
-        <v>222</v>
-      </c>
-      <c r="E82" t="s">
-        <v>123</v>
-      </c>
-      <c r="F82" t="s">
-        <v>217</v>
-      </c>
       <c r="G82" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="B83" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C83" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D83" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E83" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F83" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="G83" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
+        <v>246</v>
+      </c>
+      <c r="B84" t="s">
+        <v>247</v>
+      </c>
+      <c r="C84" t="s">
+        <v>232</v>
+      </c>
+      <c r="D84" t="s">
         <v>233</v>
       </c>
-      <c r="B84" t="s">
-        <v>234</v>
-      </c>
-      <c r="C84" t="s">
-        <v>221</v>
-      </c>
-      <c r="D84" t="s">
-        <v>222</v>
-      </c>
       <c r="E84" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F84" t="s">
+        <v>228</v>
+      </c>
+      <c r="G84" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="B85" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="C85" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D85" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E85" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F85" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="G85" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="H85" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="B86" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="C86" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D86" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E86" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F86" t="s">
+        <v>228</v>
+      </c>
+      <c r="G86" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="B87" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="C87" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D87" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E87" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F87" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="G87" t="s">
         <v>19</v>
       </c>
       <c r="H87" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="B88" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
       <c r="C88" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D88" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E88" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F88" t="s">
+        <v>228</v>
+      </c>
+      <c r="G88" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="B89" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C89" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D89" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E89" t="s">
-        <v>123</v>
+        <v>136</v>
+      </c>
+      <c r="F89" t="s">
+        <v>264</v>
+      </c>
+      <c r="G89" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
       <c r="B90" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="C90" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="D90" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E90" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F90" t="s">
-        <v>251</v>
+        <v>267</v>
       </c>
       <c r="G90" t="s">
-        <v>252</v>
+        <v>268</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="B91" t="s">
-        <v>254</v>
+        <v>270</v>
       </c>
       <c r="C91" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="D91" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="E91" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="B92" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="C92" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="D92" t="s">
         <v>37</v>
       </c>
       <c r="E92" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>259</v>
+        <v>275</v>
       </c>
       <c r="B93" t="s">
-        <v>260</v>
+        <v>276</v>
       </c>
       <c r="C93" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="D93" t="s">
-        <v>261</v>
+        <v>277</v>
       </c>
       <c r="E93" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -3112,31 +3283,31 @@
   <dimension ref="A2:B5"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="69.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.85546875" customWidth="1"/>
+    <col min="1" max="1" width="69.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:2" ht="15.75">
       <c r="A3" s="3" t="s">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:2" ht="15.75">
       <c r="A4" s="3" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="B4" s="3"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>265</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modifications for status tracker
</commit_message>
<xml_diff>
--- a/Symptom_Rootcause_Ticket_Evaluation/output/AI Jira Bug to Symptom Assignment validation.xlsx
+++ b/Symptom_Rootcause_Ticket_Evaluation/output/AI Jira Bug to Symptom Assignment validation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dentsplysirona-my.sharepoint.com/personal/christian_kurz_dentsplysirona_com/Documents/_IO-Sensor/10_Qualität/05_Feld/99_Siroforce/00_Git/Y3839-IO_Workspace/Symptom_Rootcause_Ticket_Evaluation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="164" documentId="8_{236449CA-312A-4DB1-B587-EDE847815BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A242BDD1-F3EB-4C84-8BA7-2D002368DF5A}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="8_{236449CA-312A-4DB1-B587-EDE847815BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{369355A4-1FDC-4D32-8151-CC432AB103B1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52E5B530-6EC2-40DF-B8D2-2FAAD7B66627}"/>
   </bookViews>
@@ -42,6 +42,40 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Beckhaus, Christian</author>
+  </authors>
+  <commentList>
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{019CBCAE-31FF-4FE5-AAAD-E76E64C90D45}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Beckhaus, Christian:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+ in IOSS</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
   <connection id="1" xr16:uid="{03897726-8CAB-485D-A7DD-CE652C5A5FB9}" keepAlive="1" name="Abfrage - ticket_export" description="Verbindung mit der Abfrage 'ticket_export' in der Arbeitsmappe." type="5" refreshedVersion="0" background="1">
@@ -54,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="297">
   <si>
     <t>Column1</t>
   </si>
@@ -248,6 +282,9 @@
     <t>Documentation: rotation buttons are usable</t>
   </si>
   <si>
+    <t>Software / UI Bug</t>
+  </si>
+  <si>
     <t>Y3839-304</t>
   </si>
   <si>
@@ -269,6 +306,12 @@
     <t>Sensor never becomes exposure ready when calibration file read fails</t>
   </si>
   <si>
+    <t>FW / SW Error handling</t>
+  </si>
+  <si>
+    <t>calib file corrupted</t>
+  </si>
+  <si>
     <t>Y3839-545</t>
   </si>
   <si>
@@ -302,6 +345,9 @@
     <t>Dentrix/CDR: USB3 interface fails to reconnect to sensor after multiple plug cycles, sensor LED stays orange</t>
   </si>
   <si>
+    <t>CDR not IOSS</t>
+  </si>
+  <si>
     <t>Y3839-583</t>
   </si>
   <si>
@@ -326,6 +372,12 @@
     <t>It is possible to acquire images with IOSS without enabling event detection</t>
   </si>
   <si>
+    <t>Exposure ready FW / SW bug</t>
+  </si>
+  <si>
+    <t>enables misuse</t>
+  </si>
+  <si>
     <t>Y3839-733</t>
   </si>
   <si>
@@ -692,6 +744,9 @@
     <t>No Power / "Dying Boxes" (USB module)</t>
   </si>
   <si>
+    <t>Y3839-695 has no impact to the electronic</t>
+  </si>
+  <si>
     <t>Y3839-234</t>
   </si>
   <si>
@@ -912,13 +967,25 @@
   </si>
   <si>
     <t>Prevent CDR customers to use new Firmwares (to allow interface changes)</t>
+  </si>
+  <si>
+    <t>(hidden) option to save raw images for image quality studies or bugfixing</t>
+  </si>
+  <si>
+    <t>[Y3839-737] Check for CDR Autodetect Monitor - Jira Dentsply Sirona</t>
+  </si>
+  <si>
+    <t>Log Einträge der USB Box auf dem PC verfügbar machen</t>
+  </si>
+  <si>
+    <t>IOSS Rollout via MS Store</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -940,6 +1007,27 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -958,10 +1046,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -969,8 +1058,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
@@ -1743,332 +1834,419 @@
       <c r="E16" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="F16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
         <v>54</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="F17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
         <v>54</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E18" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
         <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E19" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="F19" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
         <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="F20" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
         <v>54</v>
       </c>
       <c r="D21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E21" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="F21" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C22" t="s">
         <v>54</v>
       </c>
       <c r="D22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="F22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C23" t="s">
         <v>54</v>
       </c>
       <c r="D23" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E23" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="F23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C24" t="s">
         <v>54</v>
       </c>
       <c r="D24" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E24" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="F24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C25" t="s">
         <v>54</v>
       </c>
       <c r="D25" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E25" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="F25" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C26" t="s">
         <v>54</v>
       </c>
       <c r="D26" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E26" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="F26" t="s">
+        <v>55</v>
+      </c>
+      <c r="G26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
         <v>54</v>
       </c>
       <c r="D27" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="F27" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C28" t="s">
         <v>54</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E28" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="F28" t="s">
+        <v>55</v>
+      </c>
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+      <c r="H28" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C29" t="s">
         <v>54</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E29" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="F29" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B30" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C30" t="s">
         <v>54</v>
       </c>
       <c r="D30" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E30" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="F30" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B31" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D31" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E31" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F31" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G31" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B32" t="s">
+        <v>108</v>
+      </c>
+      <c r="C32" t="s">
         <v>102</v>
       </c>
-      <c r="C32" t="s">
-        <v>96</v>
-      </c>
       <c r="D32" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E32" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F32" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G32" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C33" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D33" t="s">
         <v>26</v>
       </c>
       <c r="E33" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F33" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G33" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B34" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C34" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D34" t="s">
         <v>26</v>
       </c>
       <c r="E34" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F34" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G34" t="s">
         <v>33</v>
@@ -2076,819 +2254,831 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B35" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C35" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D35" t="s">
         <v>26</v>
       </c>
       <c r="E35" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F35" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G35" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D36" t="s">
         <v>26</v>
       </c>
       <c r="E36" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F36" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G36" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C37" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D37" t="s">
         <v>26</v>
       </c>
       <c r="E37" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F37" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G37" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B38" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C38" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D38" t="s">
         <v>26</v>
       </c>
       <c r="E38" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F38" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G38" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B39" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C39" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D39" t="s">
         <v>26</v>
       </c>
       <c r="E39" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F39" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G39" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B40" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C40" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D40" t="s">
         <v>26</v>
       </c>
       <c r="E40" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F40" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G40" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B41" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D41" t="s">
         <v>26</v>
       </c>
       <c r="E41" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F41" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="G41" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B42" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D42" t="s">
         <v>26</v>
       </c>
       <c r="E42" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F42" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G42" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B43" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C43" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D43" t="s">
         <v>19</v>
       </c>
       <c r="E43" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F43" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G43" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C44" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D44" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E44" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B45" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C45" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E45" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" t="s">
+        <v>150</v>
+      </c>
+      <c r="B46" t="s">
+        <v>151</v>
+      </c>
+      <c r="C46" t="s">
         <v>144</v>
       </c>
-      <c r="B46" t="s">
-        <v>145</v>
-      </c>
-      <c r="C46" t="s">
-        <v>138</v>
-      </c>
       <c r="D46" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E46" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B47" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D47" t="s">
         <v>33</v>
       </c>
       <c r="E47" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B48" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C48" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D48" t="s">
         <v>33</v>
       </c>
       <c r="E48" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B49" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C49" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D49" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E49" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F49" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B50" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C50" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D50" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="E50" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F50" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G50" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:7">
       <c r="A51" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B51" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C51" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D51" t="s">
         <v>26</v>
       </c>
       <c r="E51" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F51" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B52" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C52" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D52" t="s">
         <v>26</v>
       </c>
       <c r="E52" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F52" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="53" spans="1:7">
       <c r="A53" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B53" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C53" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D53" t="s">
         <v>26</v>
       </c>
       <c r="E53" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F53" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:7">
       <c r="A54" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B54" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C54" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D54" t="s">
         <v>26</v>
       </c>
       <c r="E54" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F54" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="55" spans="1:7">
       <c r="A55" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B55" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C55" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D55" t="s">
         <v>26</v>
       </c>
       <c r="E55" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F55" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B56" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C56" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D56" t="s">
         <v>26</v>
       </c>
       <c r="E56" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F56" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G56" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B57" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C57" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D57" t="s">
         <v>26</v>
       </c>
       <c r="E57" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F57" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B58" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C58" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D58" t="s">
         <v>26</v>
       </c>
       <c r="E58" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F58" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B59" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C59" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D59" t="s">
         <v>26</v>
       </c>
       <c r="E59" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F59" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G59" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" spans="1:7">
       <c r="A60" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B60" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C60" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D60" t="s">
         <v>26</v>
       </c>
       <c r="E60" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F60" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="61" spans="1:7">
       <c r="A61" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B61" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C61" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D61" t="s">
         <v>26</v>
       </c>
       <c r="E61" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F61" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="62" spans="1:7">
       <c r="A62" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B62" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C62" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D62" t="s">
         <v>26</v>
       </c>
       <c r="E62" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F62" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="63" spans="1:7">
       <c r="A63" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B63" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C63" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D63" t="s">
         <v>26</v>
       </c>
       <c r="E63" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F63" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G63" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="64" spans="1:7">
       <c r="A64" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B64" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C64" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D64" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E64" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F64" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B65" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C65" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D65" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E65" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B66" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="C66" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D66" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E66" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F66" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G66" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B67" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C67" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D67" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E67" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F67" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="68" spans="1:7">
       <c r="A68" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B68" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C68" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D68" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E68" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B69" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C69" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D69" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E69" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B70" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C70" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D70" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E70" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B71" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C71" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D71" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="E71" t="s">
-        <v>208</v>
+        <v>214</v>
+      </c>
+      <c r="F71" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="72" spans="1:7">
       <c r="A72" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B72" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="C72" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
       </c>
       <c r="E72" t="s">
-        <v>208</v>
+        <v>214</v>
+      </c>
+      <c r="F72" t="s">
+        <v>109</v>
+      </c>
+      <c r="G72" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="B73" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C73" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="D73" t="s">
+        <v>221</v>
+      </c>
+      <c r="E73" t="s">
         <v>214</v>
       </c>
-      <c r="E73" t="s">
-        <v>208</v>
+      <c r="F73" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="74" spans="1:7">
       <c r="A74" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B74" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C74" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="D74" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E74" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B75" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C75" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D75" t="s">
         <v>26</v>
@@ -2900,18 +3090,18 @@
         <v>21</v>
       </c>
       <c r="G75" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B76" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="C76" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D76" t="s">
         <v>26</v>
@@ -2923,18 +3113,18 @@
         <v>21</v>
       </c>
       <c r="G76" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B77" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C77" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D77" t="s">
         <v>26</v>
@@ -2943,366 +3133,366 @@
         <v>27</v>
       </c>
       <c r="F77" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G77" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" t="s">
+        <v>236</v>
+      </c>
+      <c r="B78" t="s">
+        <v>237</v>
+      </c>
+      <c r="C78" t="s">
         <v>229</v>
       </c>
-      <c r="B78" t="s">
-        <v>230</v>
-      </c>
-      <c r="C78" t="s">
-        <v>222</v>
-      </c>
       <c r="D78" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="E78" t="s">
         <v>27</v>
       </c>
       <c r="F78" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G78" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B79" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C79" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D79" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E79" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F79" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G79" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" t="s">
+        <v>246</v>
+      </c>
+      <c r="B80" t="s">
+        <v>247</v>
+      </c>
+      <c r="C80" t="s">
+        <v>243</v>
+      </c>
+      <c r="D80" t="s">
+        <v>244</v>
+      </c>
+      <c r="E80" t="s">
+        <v>146</v>
+      </c>
+      <c r="F80" t="s">
         <v>239</v>
       </c>
-      <c r="B80" t="s">
-        <v>240</v>
-      </c>
-      <c r="C80" t="s">
-        <v>236</v>
-      </c>
-      <c r="D80" t="s">
-        <v>237</v>
-      </c>
-      <c r="E80" t="s">
-        <v>140</v>
-      </c>
-      <c r="F80" t="s">
-        <v>232</v>
-      </c>
       <c r="G80" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B81" t="s">
+        <v>250</v>
+      </c>
+      <c r="C81" t="s">
         <v>243</v>
       </c>
-      <c r="C81" t="s">
-        <v>236</v>
-      </c>
       <c r="D81" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E81" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F81" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G81" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
+        <v>251</v>
+      </c>
+      <c r="B82" t="s">
+        <v>252</v>
+      </c>
+      <c r="C82" t="s">
+        <v>243</v>
+      </c>
+      <c r="D82" t="s">
         <v>244</v>
       </c>
-      <c r="B82" t="s">
-        <v>245</v>
-      </c>
-      <c r="C82" t="s">
-        <v>236</v>
-      </c>
-      <c r="D82" t="s">
-        <v>237</v>
-      </c>
       <c r="E82" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F82" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G82" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B83" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C83" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D83" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E83" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F83" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G83" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="B84" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C84" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D84" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E84" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F84" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G84" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B85" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C85" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D85" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E85" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F85" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G85" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="H85" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="B86" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="C86" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D86" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E86" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F86" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G86" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B87" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C87" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D87" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E87" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F87" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="G87" t="s">
         <v>19</v>
       </c>
       <c r="H87" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B88" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C88" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D88" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E88" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F88" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G88" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B89" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C89" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D89" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E89" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F89" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="G89" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B90" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="C90" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D90" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E90" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F90" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="G90" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B91" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C91" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D91" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E91" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="B92" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="C92" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D92" t="s">
         <v>38</v>
       </c>
       <c r="E92" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B93" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="C93" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D93" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="E93" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -3315,8 +3505,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0946BBB-F06F-4E55-AF88-F61206BE9C6E}">
-  <dimension ref="A2:B5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0946BBB-F06F-4E55-AF88-F61206BE9C6E}">
+  <dimension ref="A2:B9"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="69.85546875" bestFit="1" customWidth="1"/>
@@ -3325,29 +3515,53 @@
   <sheetData>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="3" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:2" ht="15.75">
       <c r="A3" s="3" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:2" ht="15.75">
       <c r="A4" s="3" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="B4" s="3"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>285</v>
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75">
+      <c r="A6" s="3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="5" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>296</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A7" r:id="rId1" xr:uid="{1122452F-249F-424A-9BA4-F9AC9281CFA4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
add some minor changes and bugfixes
</commit_message>
<xml_diff>
--- a/Symptom_Rootcause_Ticket_Evaluation/output/AI Jira Bug to Symptom Assignment validation.xlsx
+++ b/Symptom_Rootcause_Ticket_Evaluation/output/AI Jira Bug to Symptom Assignment validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dentsplysirona-my.sharepoint.com/personal/christian_kurz_dentsplysirona_com/Documents/_IO-Sensor/10_Qualität/05_Feld/99_Siroforce/00_Git/Y3839-IO_Workspace/Symptom_Rootcause_Ticket_Evaluation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="615" documentId="8_{236449CA-312A-4DB1-B587-EDE847815BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26D658B9-0D39-435A-8CE6-98B35DD137FA}"/>
+  <xr:revisionPtr revIDLastSave="641" documentId="8_{236449CA-312A-4DB1-B587-EDE847815BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4A6E1D2-D52F-4ECF-8B93-863F5FDC64D7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52E5B530-6EC2-40DF-B8D2-2FAAD7B66627}"/>
+    <workbookView minimized="1" xWindow="4875" yWindow="1095" windowWidth="21600" windowHeight="11295" xr2:uid="{52E5B530-6EC2-40DF-B8D2-2FAAD7B66627}"/>
   </bookViews>
   <sheets>
     <sheet name="AI validation" sheetId="3" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="359">
   <si>
     <t>Column2</t>
   </si>
@@ -1155,6 +1155,18 @@
   </si>
   <si>
     <t>FW Bug</t>
+  </si>
+  <si>
+    <t>yes, but discussed with SW because issue is strongly related to a new IOSS version (arming of sensor has to be removed after a X-Ray shot -&gt; a new SetEventDetection has always be send to the interface/state 4 always necessary (checkered pattern is written in the HyperRAM) -&gt; correct signaling is reached -&gt; X-Ray is triggered =&gt; breaking changes, backward compatibility is not given any more</t>
+  </si>
+  <si>
+    <t>new FW, new IOSS and new third party SW</t>
+  </si>
+  <si>
+    <t>no, similar to 567</t>
+  </si>
+  <si>
+    <t>Christian Kurz (changed to Team_DX5)</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1269,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1269,6 +1281,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1752,30 +1765,35 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="I2" t="s">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="7" t="s">
         <v>97</v>
       </c>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2635,30 +2653,35 @@
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="A34" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="F34" s="7"/>
+      <c r="G34" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="I34" t="s">
+      <c r="H34" s="7"/>
+      <c r="I34" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="J34" t="s">
+      <c r="J34" s="7" t="s">
         <v>97</v>
       </c>
+      <c r="K34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
@@ -2911,7 +2934,7 @@
         <v>296</v>
       </c>
       <c r="J44" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="K44" t="s">
         <v>101</v>
@@ -2975,7 +2998,19 @@
         <v>34</v>
       </c>
       <c r="I46" t="s">
-        <v>296</v>
+        <v>358</v>
+      </c>
+      <c r="J46" t="s">
+        <v>101</v>
+      </c>
+      <c r="K46" t="s">
+        <v>355</v>
+      </c>
+      <c r="L46" t="s">
+        <v>270</v>
+      </c>
+      <c r="M46" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
@@ -3027,7 +3062,19 @@
         <v>34</v>
       </c>
       <c r="I48" t="s">
-        <v>296</v>
+        <v>358</v>
+      </c>
+      <c r="J48" t="s">
+        <v>357</v>
+      </c>
+      <c r="K48" t="s">
+        <v>355</v>
+      </c>
+      <c r="L48" t="s">
+        <v>270</v>
+      </c>
+      <c r="M48" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="49" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -3113,6 +3160,9 @@
       <c r="I51" t="s">
         <v>296</v>
       </c>
+      <c r="J51" t="s">
+        <v>327</v>
+      </c>
     </row>
     <row r="52" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
@@ -3537,6 +3587,9 @@
       </c>
       <c r="I67" t="s">
         <v>296</v>
+      </c>
+      <c r="J67" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>